<commit_message>
Add AEM content packages for press release, nav and footer
- Nav/footer import scripts output the logo as image + separate home link so it
  survives conversion to Universal Editor components (was an empty button)
- Header/footer blocks accept both fragment shapes (linked logo or image + link,
  bold titles with or without a wrapping paragraph)
- tools/site-package: builds a package with the Blue September press release page,
  nav, footer and their images as DAM assets
- tools/package: combines the site package and the Press Release content fragment
  package into vhi-ie-content-1.0.0.zip
- Ignore migration-work/ scratch tooling in ESLint

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-footer.report.xlsx
+++ b/tools/importer/reports/import-footer.report.xlsx
@@ -55,7 +55,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-09-29T10:44:59.771Z</t>
+    <t>2026-09-29T11:58:36.364Z</t>
   </si>
   <si>
     <t>https://www1.vhi.ie/about/media-releases-and-publications/2015/11</t>
@@ -67,7 +67,7 @@
     <t>nav</t>
   </si>
   <si>
-    <t>2026-09-29T10:13:10.419Z</t>
+    <t>2026-09-29T11:58:25.956Z</t>
   </si>
   <si>
     <t>about/media-releases-and-publications/2015/11.report.json</t>

</xml_diff>